<commit_message>
Close all non-owner and non-synology platform gaps
</commit_message>
<xml_diff>
--- a/mock-systems/excel/permit_tracker.xlsx
+++ b/mock-systems/excel/permit_tracker.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GENERAL FOLLOW UP" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DESIGN" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suppervission" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Services Provider" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PERMITOPS SYSTEM PROJECTION" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="GENERAL FOLLOW UP" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="DESIGN" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Suppervission" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Services Provider" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="PERMITOPS SYSTEM PROJECTION" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1020,17 +1020,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>R1.0</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>GHCE-APP-0142</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>WRITTEN</t>
+          <t>SEEDED</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix BD Proposal register and detail UI regressions
</commit_message>
<xml_diff>
--- a/mock-systems/excel/permit_tracker.xlsx
+++ b/mock-systems/excel/permit_tracker.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="GENERAL FOLLOW UP" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="DESIGN" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Suppervission" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Services Provider" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="PERMITOPS SYSTEM PROJECTION" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GENERAL FOLLOW UP" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DESIGN" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suppervission" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Services Provider" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PERMITOPS SYSTEM PROJECTION" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Update permit tracker workbook
</commit_message>
<xml_diff>
--- a/mock-systems/excel/permit_tracker.xlsx
+++ b/mock-systems/excel/permit_tracker.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GENERAL FOLLOW UP" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DESIGN" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suppervission" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Services Provider" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PERMITOPS SYSTEM PROJECTION" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="GENERAL FOLLOW UP" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="DESIGN" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Suppervission" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Services Provider" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="PERMITOPS SYSTEM PROJECTION" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>